<commit_message>
Workflow mapping UAT and platform comparison; document numbers and source links on records
- PO, RFQ and bill lists show the document number (PO no., RFQ no., Bill no.)
- PO record links to its RFQ; bill record links to its PO / RA bill
- mapping.js: 24 checks that every field carries correctly through procure-to-pay and
  contract-to-close (data and screen), plus data-wide invariants; final.js saves its data for it
- comparison_report.py → docs/Workflow_UAT_and_Platform_Comparison.xlsx: 28 workflow steps
  compared with ERPNext, Odoo, Zoho, Oracle Fusion, SAP S/4HANA + Ariba, with sources

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019KXwcDQC9J7A9k8nyRM74o
</commit_message>
<xml_diff>
--- a/nebullaone/docs/UAT_Report_NebullaOne.xlsx
+++ b/nebullaone/docs/UAT_Report_NebullaOne.xlsx
@@ -2824,7 +2824,7 @@
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>723 ms</t>
+          <t>745 ms</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2944,7 @@
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>6 cards, 0 tabs, 1 header buttons, loaded in 723 ms</t>
+          <t>6 cards, 0 tabs, 1 header buttons, loaded in 745 ms</t>
         </is>
       </c>
     </row>
@@ -2976,7 +2976,7 @@
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>726 ms</t>
+          <t>732 ms</t>
         </is>
       </c>
     </row>
@@ -4064,7 +4064,7 @@
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 2 tabs, 2 header buttons, loaded in 726 ms</t>
+          <t>0 cards, 2 tabs, 2 header buttons, loaded in 732 ms</t>
         </is>
       </c>
     </row>
@@ -4096,7 +4096,7 @@
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>721 ms</t>
+          <t>717 ms</t>
         </is>
       </c>
     </row>
@@ -5176,7 +5176,7 @@
       </c>
       <c r="F112" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 2 tabs, 0 header buttons, loaded in 721 ms</t>
+          <t>0 cards, 2 tabs, 0 header buttons, loaded in 717 ms</t>
         </is>
       </c>
     </row>
@@ -5208,7 +5208,7 @@
       </c>
       <c r="F113" s="3" t="inlineStr">
         <is>
-          <t>726 ms</t>
+          <t>721 ms</t>
         </is>
       </c>
     </row>
@@ -7004,7 +7004,7 @@
       </c>
       <c r="F174" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 5 tabs, 1 header buttons, loaded in 726 ms</t>
+          <t>0 cards, 5 tabs, 1 header buttons, loaded in 721 ms</t>
         </is>
       </c>
     </row>
@@ -7036,7 +7036,7 @@
       </c>
       <c r="F175" s="3" t="inlineStr">
         <is>
-          <t>743 ms</t>
+          <t>783 ms</t>
         </is>
       </c>
     </row>
@@ -7484,7 +7484,7 @@
       </c>
       <c r="F190" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 0 tabs, 1 header buttons, loaded in 743 ms</t>
+          <t>0 cards, 0 tabs, 1 header buttons, loaded in 783 ms</t>
         </is>
       </c>
     </row>
@@ -7516,7 +7516,7 @@
       </c>
       <c r="F191" s="3" t="inlineStr">
         <is>
-          <t>738 ms</t>
+          <t>759 ms</t>
         </is>
       </c>
     </row>
@@ -7714,7 +7714,7 @@
       </c>
       <c r="D198" s="3" t="inlineStr">
         <is>
-          <t>list: sort on all 4 columns</t>
+          <t>list: sort on all 5 columns</t>
         </is>
       </c>
       <c r="E198" s="4" t="inlineStr">
@@ -7742,7 +7742,7 @@
       </c>
       <c r="D199" s="3" t="inlineStr">
         <is>
-          <t>list: search "Skyline" finds rows</t>
+          <t>list: search "steel" finds rows</t>
         </is>
       </c>
       <c r="E199" s="4" t="inlineStr">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="F206" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 0 tabs, 1 header buttons, loaded in 738 ms</t>
+          <t>0 cards, 0 tabs, 1 header buttons, loaded in 759 ms</t>
         </is>
       </c>
     </row>
@@ -7996,7 +7996,7 @@
       </c>
       <c r="F207" s="3" t="inlineStr">
         <is>
-          <t>773 ms</t>
+          <t>760 ms</t>
         </is>
       </c>
     </row>
@@ -8444,7 +8444,7 @@
       </c>
       <c r="F222" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 0 tabs, 1 header buttons, loaded in 773 ms</t>
+          <t>0 cards, 0 tabs, 1 header buttons, loaded in 760 ms</t>
         </is>
       </c>
     </row>
@@ -8476,7 +8476,7 @@
       </c>
       <c r="F223" s="3" t="inlineStr">
         <is>
-          <t>755 ms</t>
+          <t>757 ms</t>
         </is>
       </c>
     </row>
@@ -8674,7 +8674,7 @@
       </c>
       <c r="D230" s="3" t="inlineStr">
         <is>
-          <t>list: sort on all 5 columns</t>
+          <t>list: sort on all 6 columns</t>
         </is>
       </c>
       <c r="E230" s="4" t="inlineStr">
@@ -8702,7 +8702,7 @@
       </c>
       <c r="D231" s="3" t="inlineStr">
         <is>
-          <t>list: search "Fe500D" finds rows</t>
+          <t>list: search "Deccan" finds rows</t>
         </is>
       </c>
       <c r="E231" s="4" t="inlineStr">
@@ -8924,7 +8924,7 @@
       </c>
       <c r="F238" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 0 tabs, 1 header buttons, loaded in 755 ms</t>
+          <t>0 cards, 0 tabs, 1 header buttons, loaded in 757 ms</t>
         </is>
       </c>
     </row>
@@ -8956,7 +8956,7 @@
       </c>
       <c r="F239" s="3" t="inlineStr">
         <is>
-          <t>809 ms</t>
+          <t>762 ms</t>
         </is>
       </c>
     </row>
@@ -9302,7 +9302,7 @@
       </c>
       <c r="D251" s="3" t="inlineStr">
         <is>
-          <t>tab "Bills": sort on all 4 columns</t>
+          <t>tab "Bills": sort on all 5 columns</t>
         </is>
       </c>
       <c r="E251" s="4" t="inlineStr">
@@ -9330,7 +9330,7 @@
       </c>
       <c r="D252" s="3" t="inlineStr">
         <is>
-          <t>tab "Bills": search "Shree" finds rows</t>
+          <t>tab "Bills": search "INV-001" finds rows</t>
         </is>
       </c>
       <c r="E252" s="4" t="inlineStr">
@@ -9340,7 +9340,7 @@
       </c>
       <c r="F252" s="3" t="inlineStr">
         <is>
-          <t>2 rows</t>
+          <t>1 rows</t>
         </is>
       </c>
     </row>
@@ -9884,7 +9884,7 @@
       </c>
       <c r="F270" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 2 tabs, 4 header buttons, loaded in 809 ms</t>
+          <t>0 cards, 2 tabs, 4 header buttons, loaded in 762 ms</t>
         </is>
       </c>
     </row>
@@ -9916,7 +9916,7 @@
       </c>
       <c r="F271" s="3" t="inlineStr">
         <is>
-          <t>773 ms</t>
+          <t>758 ms</t>
         </is>
       </c>
     </row>
@@ -10060,7 +10060,7 @@
       </c>
       <c r="F276" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 2 tabs, 0 header buttons, loaded in 773 ms</t>
+          <t>0 cards, 2 tabs, 0 header buttons, loaded in 758 ms</t>
         </is>
       </c>
     </row>
@@ -10092,7 +10092,7 @@
       </c>
       <c r="F277" s="3" t="inlineStr">
         <is>
-          <t>747 ms</t>
+          <t>749 ms</t>
         </is>
       </c>
     </row>
@@ -11128,7 +11128,7 @@
       </c>
       <c r="F312" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 3 tabs, 2 header buttons, loaded in 747 ms</t>
+          <t>0 cards, 3 tabs, 2 header buttons, loaded in 749 ms</t>
         </is>
       </c>
     </row>
@@ -11160,7 +11160,7 @@
       </c>
       <c r="F313" s="3" t="inlineStr">
         <is>
-          <t>760 ms</t>
+          <t>758 ms</t>
         </is>
       </c>
     </row>
@@ -12544,7 +12544,7 @@
       </c>
       <c r="F360" s="3" t="inlineStr">
         <is>
-          <t>4 cards, 9 tabs, 2 header buttons, loaded in 760 ms</t>
+          <t>4 cards, 9 tabs, 2 header buttons, loaded in 758 ms</t>
         </is>
       </c>
     </row>
@@ -12576,7 +12576,7 @@
       </c>
       <c r="F361" s="3" t="inlineStr">
         <is>
-          <t>765 ms</t>
+          <t>772 ms</t>
         </is>
       </c>
     </row>
@@ -12808,7 +12808,7 @@
       </c>
       <c r="F369" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 4 tabs, 1 header buttons, loaded in 765 ms</t>
+          <t>0 cards, 4 tabs, 1 header buttons, loaded in 772 ms</t>
         </is>
       </c>
     </row>
@@ -12840,7 +12840,7 @@
       </c>
       <c r="F370" s="3" t="inlineStr">
         <is>
-          <t>775 ms</t>
+          <t>771 ms</t>
         </is>
       </c>
     </row>
@@ -12960,7 +12960,7 @@
       </c>
       <c r="F374" s="3" t="inlineStr">
         <is>
-          <t>6 cards, 0 tabs, 1 header buttons, loaded in 775 ms</t>
+          <t>6 cards, 0 tabs, 1 header buttons, loaded in 771 ms</t>
         </is>
       </c>
     </row>
@@ -12992,7 +12992,7 @@
       </c>
       <c r="F375" s="3" t="inlineStr">
         <is>
-          <t>779 ms</t>
+          <t>762 ms</t>
         </is>
       </c>
     </row>
@@ -13440,7 +13440,7 @@
       </c>
       <c r="F390" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 0 tabs, 1 header buttons, loaded in 779 ms</t>
+          <t>0 cards, 0 tabs, 1 header buttons, loaded in 762 ms</t>
         </is>
       </c>
     </row>
@@ -13472,7 +13472,7 @@
       </c>
       <c r="F391" s="3" t="inlineStr">
         <is>
-          <t>755 ms</t>
+          <t>766 ms</t>
         </is>
       </c>
     </row>
@@ -13920,7 +13920,7 @@
       </c>
       <c r="F406" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 0 tabs, 1 header buttons, loaded in 755 ms</t>
+          <t>0 cards, 0 tabs, 1 header buttons, loaded in 766 ms</t>
         </is>
       </c>
     </row>
@@ -13952,7 +13952,7 @@
       </c>
       <c r="F407" s="3" t="inlineStr">
         <is>
-          <t>752 ms</t>
+          <t>755 ms</t>
         </is>
       </c>
     </row>
@@ -14428,7 +14428,7 @@
       </c>
       <c r="F423" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 0 tabs, 1 header buttons, loaded in 752 ms</t>
+          <t>0 cards, 0 tabs, 1 header buttons, loaded in 755 ms</t>
         </is>
       </c>
     </row>
@@ -14460,7 +14460,7 @@
       </c>
       <c r="F424" s="3" t="inlineStr">
         <is>
-          <t>762 ms</t>
+          <t>782 ms</t>
         </is>
       </c>
     </row>
@@ -15060,7 +15060,7 @@
       </c>
       <c r="F444" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 3 tabs, 0 header buttons, loaded in 762 ms</t>
+          <t>0 cards, 3 tabs, 0 header buttons, loaded in 782 ms</t>
         </is>
       </c>
     </row>
@@ -15092,7 +15092,7 @@
       </c>
       <c r="F445" s="3" t="inlineStr">
         <is>
-          <t>766 ms</t>
+          <t>758 ms</t>
         </is>
       </c>
     </row>
@@ -16228,7 +16228,7 @@
       </c>
       <c r="F483" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 4 tabs, 1 header buttons, loaded in 766 ms</t>
+          <t>0 cards, 4 tabs, 1 header buttons, loaded in 758 ms</t>
         </is>
       </c>
     </row>
@@ -16260,7 +16260,7 @@
       </c>
       <c r="F484" s="3" t="inlineStr">
         <is>
-          <t>758 ms</t>
+          <t>763 ms</t>
         </is>
       </c>
     </row>
@@ -17036,7 +17036,7 @@
       </c>
       <c r="F510" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 2 tabs, 1 header buttons, loaded in 758 ms</t>
+          <t>0 cards, 2 tabs, 1 header buttons, loaded in 763 ms</t>
         </is>
       </c>
     </row>
@@ -17068,7 +17068,7 @@
       </c>
       <c r="F511" s="3" t="inlineStr">
         <is>
-          <t>766 ms</t>
+          <t>749 ms</t>
         </is>
       </c>
     </row>
@@ -18232,7 +18232,7 @@
       </c>
       <c r="F550" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 3 tabs, 2 header buttons, loaded in 766 ms</t>
+          <t>0 cards, 3 tabs, 2 header buttons, loaded in 749 ms</t>
         </is>
       </c>
     </row>
@@ -18264,7 +18264,7 @@
       </c>
       <c r="F551" s="3" t="inlineStr">
         <is>
-          <t>766 ms</t>
+          <t>770 ms</t>
         </is>
       </c>
     </row>
@@ -19728,7 +19728,7 @@
       </c>
       <c r="F600" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 4 tabs, 1 header buttons, loaded in 766 ms</t>
+          <t>0 cards, 4 tabs, 1 header buttons, loaded in 770 ms</t>
         </is>
       </c>
     </row>
@@ -19760,7 +19760,7 @@
       </c>
       <c r="F601" s="3" t="inlineStr">
         <is>
-          <t>780 ms</t>
+          <t>748 ms</t>
         </is>
       </c>
     </row>
@@ -20872,7 +20872,7 @@
       </c>
       <c r="F638" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 4 tabs, 1 header buttons, loaded in 780 ms</t>
+          <t>0 cards, 4 tabs, 1 header buttons, loaded in 748 ms</t>
         </is>
       </c>
     </row>
@@ -20904,7 +20904,7 @@
       </c>
       <c r="F639" s="3" t="inlineStr">
         <is>
-          <t>763 ms</t>
+          <t>756 ms</t>
         </is>
       </c>
     </row>
@@ -21264,7 +21264,7 @@
       </c>
       <c r="F651" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 0 tabs, 0 header buttons, loaded in 763 ms</t>
+          <t>0 cards, 0 tabs, 0 header buttons, loaded in 756 ms</t>
         </is>
       </c>
     </row>
@@ -21688,7 +21688,7 @@
       </c>
       <c r="F665" s="3" t="inlineStr">
         <is>
-          <t>763 ms</t>
+          <t>755 ms</t>
         </is>
       </c>
     </row>
@@ -22012,7 +22012,7 @@
       </c>
       <c r="F676" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 2 tabs, 0 header buttons, loaded in 763 ms</t>
+          <t>0 cards, 2 tabs, 0 header buttons, loaded in 755 ms</t>
         </is>
       </c>
     </row>
@@ -22044,7 +22044,7 @@
       </c>
       <c r="F677" s="3" t="inlineStr">
         <is>
-          <t>753 ms</t>
+          <t>757 ms</t>
         </is>
       </c>
     </row>
@@ -22132,7 +22132,7 @@
       </c>
       <c r="F680" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 0 tabs, 0 header buttons, loaded in 753 ms</t>
+          <t>0 cards, 0 tabs, 0 header buttons, loaded in 757 ms</t>
         </is>
       </c>
     </row>
@@ -22164,7 +22164,7 @@
       </c>
       <c r="F681" s="3" t="inlineStr">
         <is>
-          <t>751 ms</t>
+          <t>767 ms</t>
         </is>
       </c>
     </row>
@@ -22340,7 +22340,7 @@
       </c>
       <c r="F687" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 0 tabs, 1 header buttons, loaded in 751 ms</t>
+          <t>0 cards, 0 tabs, 1 header buttons, loaded in 767 ms</t>
         </is>
       </c>
     </row>
@@ -22372,7 +22372,7 @@
       </c>
       <c r="F688" s="3" t="inlineStr">
         <is>
-          <t>757 ms</t>
+          <t>784 ms</t>
         </is>
       </c>
     </row>
@@ -22736,7 +22736,7 @@
       </c>
       <c r="F700" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 0 tabs, 0 header buttons, loaded in 757 ms</t>
+          <t>0 cards, 0 tabs, 0 header buttons, loaded in 784 ms</t>
         </is>
       </c>
     </row>
@@ -22768,7 +22768,7 @@
       </c>
       <c r="F701" s="3" t="inlineStr">
         <is>
-          <t>755 ms</t>
+          <t>760 ms</t>
         </is>
       </c>
     </row>
@@ -23388,7 +23388,7 @@
       </c>
       <c r="F722" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 0 tabs, 2 header buttons, loaded in 755 ms</t>
+          <t>0 cards, 0 tabs, 2 header buttons, loaded in 760 ms</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refreshed UAT report and UI comparison
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019KXwcDQC9J7A9k8nyRM74o
</commit_message>
<xml_diff>
--- a/nebullaone/docs/UAT_Report_NebullaOne.xlsx
+++ b/nebullaone/docs/UAT_Report_NebullaOne.xlsx
@@ -2816,7 +2816,7 @@
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>746 ms</t>
+          <t>731 ms</t>
         </is>
       </c>
     </row>
@@ -3904,7 +3904,7 @@
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 2 tabs, 2 header buttons, loaded in 746 ms</t>
+          <t>0 cards, 2 tabs, 2 header buttons, loaded in 731 ms</t>
         </is>
       </c>
     </row>
@@ -3936,7 +3936,7 @@
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>720 ms</t>
+          <t>722 ms</t>
         </is>
       </c>
     </row>
@@ -5016,7 +5016,7 @@
       </c>
       <c r="F112" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 2 tabs, 0 header buttons, loaded in 720 ms</t>
+          <t>0 cards, 2 tabs, 0 header buttons, loaded in 722 ms</t>
         </is>
       </c>
     </row>
@@ -5048,7 +5048,7 @@
       </c>
       <c r="F113" s="3" t="inlineStr">
         <is>
-          <t>752 ms</t>
+          <t>732 ms</t>
         </is>
       </c>
     </row>
@@ -6844,7 +6844,7 @@
       </c>
       <c r="F174" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 5 tabs, 1 header buttons, loaded in 752 ms</t>
+          <t>0 cards, 5 tabs, 1 header buttons, loaded in 732 ms</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="F175" s="3" t="inlineStr">
         <is>
-          <t>775 ms</t>
+          <t>724 ms</t>
         </is>
       </c>
     </row>
@@ -7324,7 +7324,7 @@
       </c>
       <c r="F190" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 0 tabs, 1 header buttons, loaded in 775 ms</t>
+          <t>0 cards, 0 tabs, 1 header buttons, loaded in 724 ms</t>
         </is>
       </c>
     </row>
@@ -7356,7 +7356,7 @@
       </c>
       <c r="F191" s="3" t="inlineStr">
         <is>
-          <t>756 ms</t>
+          <t>721 ms</t>
         </is>
       </c>
     </row>
@@ -7804,7 +7804,7 @@
       </c>
       <c r="F206" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 0 tabs, 1 header buttons, loaded in 756 ms</t>
+          <t>0 cards, 0 tabs, 1 header buttons, loaded in 721 ms</t>
         </is>
       </c>
     </row>
@@ -7836,7 +7836,7 @@
       </c>
       <c r="F207" s="3" t="inlineStr">
         <is>
-          <t>767 ms</t>
+          <t>744 ms</t>
         </is>
       </c>
     </row>
@@ -8284,7 +8284,7 @@
       </c>
       <c r="F222" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 0 tabs, 1 header buttons, loaded in 767 ms</t>
+          <t>0 cards, 0 tabs, 1 header buttons, loaded in 744 ms</t>
         </is>
       </c>
     </row>
@@ -8316,7 +8316,7 @@
       </c>
       <c r="F223" s="3" t="inlineStr">
         <is>
-          <t>759 ms</t>
+          <t>723 ms</t>
         </is>
       </c>
     </row>
@@ -8792,7 +8792,7 @@
       </c>
       <c r="F239" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 0 tabs, 1 header buttons, loaded in 759 ms</t>
+          <t>0 cards, 0 tabs, 1 header buttons, loaded in 723 ms</t>
         </is>
       </c>
     </row>
@@ -8824,7 +8824,7 @@
       </c>
       <c r="F240" s="3" t="inlineStr">
         <is>
-          <t>757 ms</t>
+          <t>750 ms</t>
         </is>
       </c>
     </row>
@@ -9752,7 +9752,7 @@
       </c>
       <c r="F271" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 2 tabs, 4 header buttons, loaded in 757 ms</t>
+          <t>0 cards, 2 tabs, 4 header buttons, loaded in 750 ms</t>
         </is>
       </c>
     </row>
@@ -9784,7 +9784,7 @@
       </c>
       <c r="F272" s="3" t="inlineStr">
         <is>
-          <t>777 ms</t>
+          <t>757 ms</t>
         </is>
       </c>
     </row>
@@ -9928,7 +9928,7 @@
       </c>
       <c r="F277" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 2 tabs, 0 header buttons, loaded in 777 ms</t>
+          <t>0 cards, 2 tabs, 0 header buttons, loaded in 757 ms</t>
         </is>
       </c>
     </row>
@@ -9960,7 +9960,7 @@
       </c>
       <c r="F278" s="3" t="inlineStr">
         <is>
-          <t>754 ms</t>
+          <t>771 ms</t>
         </is>
       </c>
     </row>
@@ -10996,7 +10996,7 @@
       </c>
       <c r="F313" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 3 tabs, 2 header buttons, loaded in 754 ms</t>
+          <t>0 cards, 3 tabs, 2 header buttons, loaded in 771 ms</t>
         </is>
       </c>
     </row>
@@ -11028,7 +11028,7 @@
       </c>
       <c r="F314" s="3" t="inlineStr">
         <is>
-          <t>756 ms</t>
+          <t>774 ms</t>
         </is>
       </c>
     </row>
@@ -12412,7 +12412,7 @@
       </c>
       <c r="F361" s="3" t="inlineStr">
         <is>
-          <t>4 cards, 9 tabs, 2 header buttons, loaded in 756 ms</t>
+          <t>4 cards, 9 tabs, 2 header buttons, loaded in 774 ms</t>
         </is>
       </c>
     </row>
@@ -12444,7 +12444,7 @@
       </c>
       <c r="F362" s="3" t="inlineStr">
         <is>
-          <t>766 ms</t>
+          <t>777 ms</t>
         </is>
       </c>
     </row>
@@ -12676,7 +12676,7 @@
       </c>
       <c r="F370" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 4 tabs, 1 header buttons, loaded in 766 ms</t>
+          <t>0 cards, 4 tabs, 1 header buttons, loaded in 777 ms</t>
         </is>
       </c>
     </row>
@@ -12708,7 +12708,7 @@
       </c>
       <c r="F371" s="3" t="inlineStr">
         <is>
-          <t>784 ms</t>
+          <t>776 ms</t>
         </is>
       </c>
     </row>
@@ -12828,7 +12828,7 @@
       </c>
       <c r="F375" s="3" t="inlineStr">
         <is>
-          <t>6 cards, 0 tabs, 1 header buttons, loaded in 784 ms</t>
+          <t>6 cards, 0 tabs, 1 header buttons, loaded in 776 ms</t>
         </is>
       </c>
     </row>
@@ -12860,7 +12860,7 @@
       </c>
       <c r="F376" s="3" t="inlineStr">
         <is>
-          <t>777 ms</t>
+          <t>764 ms</t>
         </is>
       </c>
     </row>
@@ -13308,7 +13308,7 @@
       </c>
       <c r="F391" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 0 tabs, 1 header buttons, loaded in 777 ms</t>
+          <t>0 cards, 0 tabs, 1 header buttons, loaded in 764 ms</t>
         </is>
       </c>
     </row>
@@ -13340,7 +13340,7 @@
       </c>
       <c r="F392" s="3" t="inlineStr">
         <is>
-          <t>795 ms</t>
+          <t>768 ms</t>
         </is>
       </c>
     </row>
@@ -13788,7 +13788,7 @@
       </c>
       <c r="F407" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 0 tabs, 1 header buttons, loaded in 795 ms</t>
+          <t>0 cards, 0 tabs, 1 header buttons, loaded in 768 ms</t>
         </is>
       </c>
     </row>
@@ -13820,7 +13820,7 @@
       </c>
       <c r="F408" s="3" t="inlineStr">
         <is>
-          <t>769 ms</t>
+          <t>760 ms</t>
         </is>
       </c>
     </row>
@@ -14296,7 +14296,7 @@
       </c>
       <c r="F424" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 0 tabs, 1 header buttons, loaded in 769 ms</t>
+          <t>0 cards, 0 tabs, 1 header buttons, loaded in 760 ms</t>
         </is>
       </c>
     </row>
@@ -14328,7 +14328,7 @@
       </c>
       <c r="F425" s="3" t="inlineStr">
         <is>
-          <t>755 ms</t>
+          <t>752 ms</t>
         </is>
       </c>
     </row>
@@ -14928,7 +14928,7 @@
       </c>
       <c r="F445" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 3 tabs, 0 header buttons, loaded in 755 ms</t>
+          <t>0 cards, 3 tabs, 0 header buttons, loaded in 752 ms</t>
         </is>
       </c>
     </row>
@@ -14960,7 +14960,7 @@
       </c>
       <c r="F446" s="3" t="inlineStr">
         <is>
-          <t>766 ms</t>
+          <t>759 ms</t>
         </is>
       </c>
     </row>
@@ -16096,7 +16096,7 @@
       </c>
       <c r="F484" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 4 tabs, 1 header buttons, loaded in 766 ms</t>
+          <t>0 cards, 4 tabs, 1 header buttons, loaded in 759 ms</t>
         </is>
       </c>
     </row>
@@ -16128,7 +16128,7 @@
       </c>
       <c r="F485" s="3" t="inlineStr">
         <is>
-          <t>760 ms</t>
+          <t>761 ms</t>
         </is>
       </c>
     </row>
@@ -16904,7 +16904,7 @@
       </c>
       <c r="F511" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 2 tabs, 1 header buttons, loaded in 760 ms</t>
+          <t>0 cards, 2 tabs, 1 header buttons, loaded in 761 ms</t>
         </is>
       </c>
     </row>
@@ -16936,7 +16936,7 @@
       </c>
       <c r="F512" s="3" t="inlineStr">
         <is>
-          <t>777 ms</t>
+          <t>776 ms</t>
         </is>
       </c>
     </row>
@@ -18100,7 +18100,7 @@
       </c>
       <c r="F551" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 3 tabs, 2 header buttons, loaded in 777 ms</t>
+          <t>0 cards, 3 tabs, 2 header buttons, loaded in 776 ms</t>
         </is>
       </c>
     </row>
@@ -18132,7 +18132,7 @@
       </c>
       <c r="F552" s="3" t="inlineStr">
         <is>
-          <t>783 ms</t>
+          <t>778 ms</t>
         </is>
       </c>
     </row>
@@ -19596,7 +19596,7 @@
       </c>
       <c r="F601" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 4 tabs, 1 header buttons, loaded in 783 ms</t>
+          <t>0 cards, 4 tabs, 1 header buttons, loaded in 778 ms</t>
         </is>
       </c>
     </row>
@@ -19628,7 +19628,7 @@
       </c>
       <c r="F602" s="3" t="inlineStr">
         <is>
-          <t>774 ms</t>
+          <t>767 ms</t>
         </is>
       </c>
     </row>
@@ -20740,7 +20740,7 @@
       </c>
       <c r="F639" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 4 tabs, 1 header buttons, loaded in 774 ms</t>
+          <t>0 cards, 4 tabs, 1 header buttons, loaded in 767 ms</t>
         </is>
       </c>
     </row>
@@ -20772,7 +20772,7 @@
       </c>
       <c r="F640" s="3" t="inlineStr">
         <is>
-          <t>766 ms</t>
+          <t>757 ms</t>
         </is>
       </c>
     </row>
@@ -21132,7 +21132,7 @@
       </c>
       <c r="F652" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 0 tabs, 0 header buttons, loaded in 766 ms</t>
+          <t>0 cards, 0 tabs, 0 header buttons, loaded in 757 ms</t>
         </is>
       </c>
     </row>
@@ -21164,7 +21164,7 @@
       </c>
       <c r="F653" s="3" t="inlineStr">
         <is>
-          <t>757 ms</t>
+          <t>755 ms</t>
         </is>
       </c>
     </row>
@@ -21524,7 +21524,7 @@
       </c>
       <c r="F665" s="3" t="inlineStr">
         <is>
-          <t>4 cards, 0 tabs, 0 header buttons, loaded in 757 ms</t>
+          <t>4 cards, 0 tabs, 0 header buttons, loaded in 755 ms</t>
         </is>
       </c>
     </row>
@@ -21556,7 +21556,7 @@
       </c>
       <c r="F666" s="3" t="inlineStr">
         <is>
-          <t>757 ms</t>
+          <t>758 ms</t>
         </is>
       </c>
     </row>
@@ -21880,7 +21880,7 @@
       </c>
       <c r="F677" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 2 tabs, 0 header buttons, loaded in 757 ms</t>
+          <t>0 cards, 2 tabs, 0 header buttons, loaded in 758 ms</t>
         </is>
       </c>
     </row>
@@ -21912,7 +21912,7 @@
       </c>
       <c r="F678" s="3" t="inlineStr">
         <is>
-          <t>760 ms</t>
+          <t>759 ms</t>
         </is>
       </c>
     </row>
@@ -22000,7 +22000,7 @@
       </c>
       <c r="F681" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 0 tabs, 0 header buttons, loaded in 760 ms</t>
+          <t>0 cards, 0 tabs, 0 header buttons, loaded in 759 ms</t>
         </is>
       </c>
     </row>
@@ -22032,7 +22032,7 @@
       </c>
       <c r="F682" s="3" t="inlineStr">
         <is>
-          <t>754 ms</t>
+          <t>756 ms</t>
         </is>
       </c>
     </row>
@@ -22208,7 +22208,7 @@
       </c>
       <c r="F688" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 0 tabs, 1 header buttons, loaded in 754 ms</t>
+          <t>0 cards, 0 tabs, 1 header buttons, loaded in 756 ms</t>
         </is>
       </c>
     </row>
@@ -22240,7 +22240,7 @@
       </c>
       <c r="F689" s="3" t="inlineStr">
         <is>
-          <t>772 ms</t>
+          <t>751 ms</t>
         </is>
       </c>
     </row>
@@ -22604,7 +22604,7 @@
       </c>
       <c r="F701" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 0 tabs, 0 header buttons, loaded in 772 ms</t>
+          <t>0 cards, 0 tabs, 0 header buttons, loaded in 751 ms</t>
         </is>
       </c>
     </row>
@@ -22636,7 +22636,7 @@
       </c>
       <c r="F702" s="3" t="inlineStr">
         <is>
-          <t>756 ms</t>
+          <t>801 ms</t>
         </is>
       </c>
     </row>
@@ -23256,7 +23256,7 @@
       </c>
       <c r="F723" s="3" t="inlineStr">
         <is>
-          <t>0 cards, 0 tabs, 2 header buttons, loaded in 756 ms</t>
+          <t>0 cards, 0 tabs, 2 header buttons, loaded in 801 ms</t>
         </is>
       </c>
     </row>

</xml_diff>